<commit_message>
Test ajout attribut 8968e4ca61d17c5205f92aeb86fe90ce0c04d37d
</commit_message>
<xml_diff>
--- a/test-dan/ig/StructureDefinition-Professionnel.xlsx
+++ b/test-dan/ig/StructureDefinition-Professionnel.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="126">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-12T13:42:24+00:00</t>
+    <t>2026-03-12T13:48:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -327,6 +327,15 @@
   </si>
   <si>
     <t>Boîte(s) aux lettres du service de messagerie sécurisée de santé (MSS) rattachée(s) au professionnel.</t>
+  </si>
+  <si>
+    <t>Professionnel.attributTest</t>
+  </si>
+  <si>
+    <t>Libellé définition</t>
+  </si>
+  <si>
+    <t>Libellé short</t>
   </si>
   <si>
     <t>Professionnel.ExerciceProfessionnel</t>
@@ -698,7 +707,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ17"/>
+  <dimension ref="A1:AJ18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.9609375" customWidth="true" bestFit="true"/>
@@ -1762,7 +1771,7 @@
         <v>72</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>71</v>
@@ -1774,10 +1783,10 @@
         <v>71</v>
       </c>
       <c r="K11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="L11" t="s" s="2">
         <v>103</v>
-      </c>
-      <c r="L11" t="s" s="2">
-        <v>104</v>
       </c>
       <c r="M11" t="s" s="2">
         <v>104</v>
@@ -1837,7 +1846,7 @@
         <v>72</v>
       </c>
       <c r="AH11" t="s" s="2">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="AI11" t="s" s="2">
         <v>71</v>
@@ -2443,6 +2452,106 @@
         <v>71</v>
       </c>
       <c r="AJ17" t="s" s="2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="B18" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" t="s" s="2">
+        <v>72</v>
+      </c>
+      <c r="G18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="H18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="I18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="J18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="K18" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="L18" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="M18" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="R18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="S18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="T18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="U18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="V18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="W18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="X18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="Y18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="Z18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AA18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AB18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AC18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AD18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AE18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AF18" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>72</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
         <v>71</v>
       </c>
     </row>

</xml_diff>